<commit_message>
Proposte intitolazioni future + pulizia file obsoleti
Aggiornamenti:
- F_M DATE.xlsx: aggiunte 5 persone proposte nel foglio DONNE
  (Rina Monti, Margherita Hack, Ada Buffulini, Maria Dalle Donne,
   Alessandro Zijno) con dati biografici completi
- bologna_KG_corretto.ttl: aggiunte le 5 persone come cpv:Person
  con ex:proposta "true" (6803 triple totali, +20 rispetto a prima)
- proposte_intitolazioni_future.csv: aggiunto dal branch main

Eliminati file obsoleti/duplicati:
- bologna_KG_definitivo.ttl (sostituito da bologna_KG_corretto.ttl)
- bologna_entita_uniche.csv (duplicato di bologna_entita_uniche_comma.csv)
- bologna_gender_gap.ttl (TTL non corretto: cpv:sex sempre Male)
- bologna_grafo.ttl (TTL non corretto: cpv:sex assente)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/F_M DATE.xlsx
+++ b/F_M DATE.xlsx
@@ -30514,7 +30514,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E125"/>
+  <dimension ref="A1:E130"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="22.38" customWidth="1" style="10" min="1" max="1"/>
@@ -32755,6 +32755,141 @@
       <c r="E125" s="0" t="inlineStr">
         <is>
           <t>16 maggio 1894, Roma</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Rina Monti (Cesarina Monti Stella)</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Biologa, zoologa, limnologa; professoressa ordinaria di Zoologia e Anatomia Comparata</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>16 agosto 1871, Arcisate (VA)</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>25 gennaio 1937, Pavia</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Margherita Hack</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Astrofisica, accademica, divulgatrice scientifica, attivista</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>12 giugno 1922, Firenze</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>29 giugno 2013, Trieste</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Ada Buffulini</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Medico (radiologa), partigiana, organizzatrice della resistenza interna nel campo di transito di Bolzano</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>28 settembre 1912, Trieste</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>3 luglio 1991, Milano</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Maria Dalle Donne (Maria Carolina Nanni Dalle Donne, anche Anna Maria Dalle Donne)</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Medico, ginecologa, accademica; Direttrice della Scuola di Ostetricia di Bologna</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>12 luglio 1778, Roncastaldo di Loiano (BO)</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>9 gennaio 1842, Bologna</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Alessandro Zijno (detta 'l'Ambigua')</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Attivista transfemminista e queer; fondatrice del Laboratorio Smaschieramenti – Atlantide di Bologna</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>data non reperita</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>17 settembre 2011, Bologna (Hospice Bellaria)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: rimosse proposte future da F_M DATE.xlsx
Le 5 persone proposte (Rina Monti, Margherita Hack, Ada Buffulini,
Maria Dalle Donne, Alessandro Zijno) non vanno nel file biografico
delle dediche esistenti — restano in proposte_intitolazioni_future.csv
e nel KG come cpv:Person con ex:proposta true.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/F_M DATE.xlsx
+++ b/F_M DATE.xlsx
@@ -30514,7 +30514,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E130"/>
+  <dimension ref="A1:E125"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="22.38" customWidth="1" style="10" min="1" max="1"/>
@@ -32755,141 +32755,6 @@
       <c r="E125" s="0" t="inlineStr">
         <is>
           <t>16 maggio 1894, Roma</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>Rina Monti (Cesarina Monti Stella)</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>Biologa, zoologa, limnologa; professoressa ordinaria di Zoologia e Anatomia Comparata</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>16 agosto 1871, Arcisate (VA)</t>
-        </is>
-      </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>25 gennaio 1937, Pavia</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>Margherita Hack</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>Astrofisica, accademica, divulgatrice scientifica, attivista</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>12 giugno 1922, Firenze</t>
-        </is>
-      </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>29 giugno 2013, Trieste</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>Ada Buffulini</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>Medico (radiologa), partigiana, organizzatrice della resistenza interna nel campo di transito di Bolzano</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>28 settembre 1912, Trieste</t>
-        </is>
-      </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>3 luglio 1991, Milano</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>Maria Dalle Donne (Maria Carolina Nanni Dalle Donne, anche Anna Maria Dalle Donne)</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>Medico, ginecologa, accademica; Direttrice della Scuola di Ostetricia di Bologna</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>12 luglio 1778, Roncastaldo di Loiano (BO)</t>
-        </is>
-      </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>9 gennaio 1842, Bologna</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>Alessandro Zijno (detta 'l'Ambigua')</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>Attivista transfemminista e queer; fondatrice del Laboratorio Smaschieramenti – Atlantide di Bologna</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>data non reperita</t>
-        </is>
-      </c>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t>17 settembre 2011, Bologna (Hospice Bellaria)</t>
         </is>
       </c>
     </row>

</xml_diff>